<commit_message>
Add 3 blog posts (calendar blogs 4-6) + mark done in tracker
- The 12 Questions Every Indian Investor Will Ask Before Series A (May 28)
- What Operators Actually Do in a Startup vs Advisors and Mentors (May 29)
- How to Scale a D2C Brand in India from Rs1 Cr to Rs10 Cr ARR (May 29)
- Regenerate blog manifest (34 posts)
- Mark blogs 4-6 as done in 180-day calendar xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maxinor_180Day_Deduped_v2.xlsx
+++ b/Maxinor_180Day_Deduped_v2.xlsx
@@ -1934,7 +1934,7 @@
       </c>
       <c r="K7" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="K8" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="K9" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 2 blog posts (calendar blogs 7-8) + mark done in tracker
- The Maxinor Execution Ladder: 5 Levels Every Startup Must Climb (May 31)
- Why Fractional CMOs Outperform Full-Time Hires for Indian Startups (Jun 1)
- Regenerate blog manifest (36 posts)
- Mark blogs 7-8 as done in 180-day calendar xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maxinor_180Day_Deduped_v2.xlsx
+++ b/Maxinor_180Day_Deduped_v2.xlsx
@@ -2087,7 +2087,7 @@
       </c>
       <c r="K10" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="K11" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish blog #9: AI-Native Company Building India 2026
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maxinor_180Day_Deduped_v2.xlsx
+++ b/Maxinor_180Day_Deduped_v2.xlsx
@@ -2087,7 +2087,7 @@
       </c>
       <c r="K10" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="K11" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="K12" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AIO/GEO/AEO fixes + 2 new blogs (14-15)
AIO/GEO/AEO:
- robots.ts: add all AI crawlers (GPTBot, ClaudeBot, PerplexityBot, OAI-SearchBot, etc.) + fix sitemap URLs
- layout.tsx: add Organization + WebSite JSON-LD schema sitewide
- blog/[slug]/page.tsx: add BreadcrumbList schema, Person knowsAbout + sameAs, semantic <time> tags, visible dateModified
- llms.txt: fix URLs to correct basePath, remove em dash, update blog list to 20+ posts grouped by topic
- build/page.tsx: add FAQPage schema + visible FAQ section
- scale/page.tsx: add FAQPage schema + visible FAQ section
- capability-centre/page.tsx: add FAQPage schema + visible FAQ section

Blogs:
- Blog 14: What Investors Actually Look for in Indian Startups (Jun 8)
- Blog 15: FinTech Startup Scaling Playbook India 2026 (Jun 8)
- Manifest regenerated (43 posts)
- Tracker updated (blogs 14-15 marked done)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maxinor_180Day_Deduped_v2.xlsx
+++ b/Maxinor_180Day_Deduped_v2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="✅ Existing Blogs Audit" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📅 180-Day Calendar (Deduped)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="📊 Summary &amp; Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ Existing Blogs Audit" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 180-Day Calendar (Deduped)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Summary &amp; Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="K18" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AIO/GEO/AEO fixes + publish blogs 14-15 to main
- robots.ts: all AI crawlers declared, sitemap URLs fixed
- layout.tsx: Organization + WebSite schema sitewide
- blog posts: BreadcrumbList + Person schema, semantic time tags
- llms.txt: correct URLs, updated blog list
- build/scale/capability-centre: FAQPage schema + visible FAQ sections
- Blog 14: What Investors Actually Look for in Indian Startups
- Blog 15: FinTech Startup Scaling Playbook India 2026

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maxinor_180Day_Deduped_v2.xlsx
+++ b/Maxinor_180Day_Deduped_v2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="✅ Existing Blogs Audit" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📅 180-Day Calendar (Deduped)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="📊 Summary &amp; Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ Existing Blogs Audit" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 180-Day Calendar (Deduped)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Summary &amp; Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2444,7 +2444,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="K18" s="28" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>✅ Done</t>
         </is>
       </c>
     </row>

</xml_diff>